<commit_message>
Align sanitized fixture with official LEA long format
</commit_message>
<xml_diff>
--- a/tests/Fixtures/lea_prices_valid.xlsx
+++ b/tests/Fixtures/lea_prices_valid.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEA duomenys" sheetId="1" r:id="R833fbba9d685435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Degalų kainos" sheetId="1" r:id="R4f6a5682b0f940f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,8 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0.000"/>
+    <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -90,7 +91,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -108,13 +109,16 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -317,13 +321,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="48.11000061035156" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -335,138 +338,283 @@
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
       <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="6" t="str">
+    </x:row>
+    <x:row r="2"/>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="6" t="str">
         <x:v>Tik automatinėms patikroms — visi pavadinimai ir adresai išgalvoti</x:v>
       </x:c>
-      <x:c r="B2" s="6"/>
-      <x:c r="C2" s="6"/>
-      <x:c r="D2" s="6"/>
-      <x:c r="E2" s="6"/>
-      <x:c r="F2" s="6"/>
-      <x:c r="G2" s="6"/>
-    </x:row>
-    <x:row r="3" ht="38" hidden="0" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>Įmonė</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="str">
-        <x:v>Vieta (savivaldybė)</x:v>
-      </x:c>
-      <x:c r="C3" s="11" t="str">
-        <x:v>Vieta (gyvenvietė, gatvė)</x:v>
-      </x:c>
-      <x:c r="D3" s="11" t="str">
-        <x:v>Pb 95</x:v>
-      </x:c>
-      <x:c r="E3" s="11" t="str">
-        <x:v>Pb 98</x:v>
-      </x:c>
-      <x:c r="F3" s="11" t="str">
-        <x:v>Dyzelinas</x:v>
-      </x:c>
-      <x:c r="G3" s="11" t="str">
-        <x:v>Suskystintos naftos dujos</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="12" t="str">
-        <x:v>Circle K</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>Vilniaus m. sav.</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
-        <x:v>Vilnius, Testų g. 1</x:v>
-      </x:c>
-      <x:c r="D4" s="13" t="n">
-        <x:v>1.499</x:v>
-      </x:c>
-      <x:c r="E4" s="13" t="n">
-        <x:v>1.599</x:v>
-      </x:c>
-      <x:c r="F4" s="13" t="n">
-        <x:v>1.399</x:v>
-      </x:c>
-      <x:c r="G4" s="13" t="n">
-        <x:v>0.699</x:v>
-      </x:c>
-    </x:row>
+      <x:c r="B3" s="6"/>
+      <x:c r="C3" s="6"/>
+      <x:c r="D3" s="6"/>
+      <x:c r="E3" s="6"/>
+      <x:c r="F3" s="6"/>
+    </x:row>
+    <x:row r="4"/>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
+        <x:v>Įmonė</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Savivaldybė</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Adresas</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>Degalų tipas</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>Kaina (EUR/l)</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>Pateikimo data</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="13" t="str">
+        <x:v>Circle K</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="str">
+        <x:v>Vilniaus m. sav.</x:v>
+      </x:c>
+      <x:c r="C6" s="13" t="str">
+        <x:v>Vilnius, Testų g. 1</x:v>
+      </x:c>
+      <x:c r="D6" s="13" t="str">
+        <x:v>Dyzelinas</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="n">
+        <x:v>1.399</x:v>
+      </x:c>
+      <x:c r="F6" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="13" t="str">
+        <x:v>Circle K</x:v>
+      </x:c>
+      <x:c r="B7" s="13" t="str">
+        <x:v>Vilniaus m. sav.</x:v>
+      </x:c>
+      <x:c r="C7" s="13" t="str">
+        <x:v>Vilnius, Testų g. 1</x:v>
+      </x:c>
+      <x:c r="D7" s="13" t="str">
+        <x:v>95 benzinas</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="n">
+        <x:v>1.499</x:v>
+      </x:c>
+      <x:c r="F7" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="13" t="str">
+        <x:v>Circle K</x:v>
+      </x:c>
+      <x:c r="B8" s="13" t="str">
+        <x:v>Vilniaus m. sav.</x:v>
+      </x:c>
+      <x:c r="C8" s="13" t="str">
+        <x:v>Vilnius, Testų g. 1</x:v>
+      </x:c>
+      <x:c r="D8" s="13" t="str">
+        <x:v>SND</x:v>
+      </x:c>
+      <x:c r="E8" s="14" t="n">
+        <x:v>0.699</x:v>
+      </x:c>
+      <x:c r="F8" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="13" t="str">
         <x:v>Viada</x:v>
       </x:c>
-      <x:c r="B5" s="12" t="str">
+      <x:c r="B9" s="13" t="str">
         <x:v>Kauno m. sav.</x:v>
       </x:c>
-      <x:c r="C5" s="12" t="str">
+      <x:c r="C9" s="13" t="str">
         <x:v>Kaunas, Pavyzdžio pr. 2</x:v>
       </x:c>
-      <x:c r="D5" s="13" t="n">
+      <x:c r="D9" s="13" t="str">
+        <x:v>Dyzelinas</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="n">
+        <x:v>1.409</x:v>
+      </x:c>
+      <x:c r="F9" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="13" t="str">
+        <x:v>Viada</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="str">
+        <x:v>Kauno m. sav.</x:v>
+      </x:c>
+      <x:c r="C10" s="13" t="str">
+        <x:v>Kaunas, Pavyzdžio pr. 2</x:v>
+      </x:c>
+      <x:c r="D10" s="13" t="str">
+        <x:v>95 benzinas</x:v>
+      </x:c>
+      <x:c r="E10" s="14" t="n">
         <x:v>1.509</x:v>
       </x:c>
-      <x:c r="E5" s="13" t="n">
-        <x:v>1.609</x:v>
-      </x:c>
-      <x:c r="F5" s="13" t="n">
-        <x:v>1.409</x:v>
-      </x:c>
-      <x:c r="G5" s="13" t="n">
+      <x:c r="F10" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="13" t="str">
+        <x:v>Viada</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="str">
+        <x:v>Kauno m. sav.</x:v>
+      </x:c>
+      <x:c r="C11" s="13" t="str">
+        <x:v>Kaunas, Pavyzdžio pr. 2</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="str">
+        <x:v>SND</x:v>
+      </x:c>
+      <x:c r="E11" s="14" t="n">
         <x:v>0.709</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="12" t="str">
+      <x:c r="F11" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="13" t="str">
         <x:v>Neste</x:v>
       </x:c>
-      <x:c r="B6" s="12" t="str">
+      <x:c r="B12" s="13" t="str">
         <x:v>Klaipėdos m. sav.</x:v>
       </x:c>
-      <x:c r="C6" s="12" t="str">
+      <x:c r="C12" s="13" t="str">
         <x:v>Klaipėda, Bandymų g. 3</x:v>
       </x:c>
-      <x:c r="D6" s="13" t="n">
+      <x:c r="D12" s="13" t="str">
+        <x:v>Dyzelinas</x:v>
+      </x:c>
+      <x:c r="E12" s="14" t="n">
+        <x:v>1.419</x:v>
+      </x:c>
+      <x:c r="F12" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="13" t="str">
+        <x:v>Neste</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>Klaipėdos m. sav.</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>Klaipėda, Bandymų g. 3</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>95 benzinas</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="n">
         <x:v>1.519</x:v>
       </x:c>
-      <x:c r="E6" s="13" t="n">
-        <x:v>1.619</x:v>
-      </x:c>
-      <x:c r="F6" s="13" t="n">
-        <x:v>1.419</x:v>
-      </x:c>
-      <x:c r="G6" s="13" t="n">
+      <x:c r="F13" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="13" t="str">
+        <x:v>Neste</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>Klaipėdos m. sav.</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>Klaipėda, Bandymų g. 3</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="str">
+        <x:v>SND</x:v>
+      </x:c>
+      <x:c r="E14" s="14" t="n">
         <x:v>0.719</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="14" t="str">
+      <x:c r="F14" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="13" t="str">
         <x:v>Orlen</x:v>
       </x:c>
-      <x:c r="B7" s="14" t="str">
+      <x:c r="B15" s="13" t="str">
         <x:v>Šiaulių m. sav.</x:v>
       </x:c>
-      <x:c r="C7" s="14" t="str">
+      <x:c r="C15" s="13" t="str">
         <x:v>Šiauliai, Sintetinė g. 4</x:v>
       </x:c>
-      <x:c r="D7" s="15" t="n">
+      <x:c r="D15" s="13" t="str">
+        <x:v>Dyzelinas</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="n">
+        <x:v>1.429</x:v>
+      </x:c>
+      <x:c r="F15" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="13" t="str">
+        <x:v>Orlen</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>Šiaulių m. sav.</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>Šiauliai, Sintetinė g. 4</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>95 benzinas</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="n">
         <x:v>1.529</x:v>
       </x:c>
-      <x:c r="E7" s="15" t="n">
-        <x:v>1.629</x:v>
-      </x:c>
-      <x:c r="F7" s="15" t="n">
-        <x:v>1.429</x:v>
-      </x:c>
-      <x:c r="G7" s="15" t="n">
+      <x:c r="F16" s="15" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="16" t="str">
+        <x:v>Orlen</x:v>
+      </x:c>
+      <x:c r="B17" s="16" t="str">
+        <x:v>Šiaulių m. sav.</x:v>
+      </x:c>
+      <x:c r="C17" s="16" t="str">
+        <x:v>Šiauliai, Sintetinė g. 4</x:v>
+      </x:c>
+      <x:c r="D17" s="16" t="str">
+        <x:v>SND</x:v>
+      </x:c>
+      <x:c r="E17" s="17" t="n">
         <x:v>0.729</x:v>
+      </x:c>
+      <x:c r="F17" s="18" t="n">
+        <x:v>46220</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
-    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>